<commit_message>
theme name,icon change,login,export toast error fix, ip not displayed fix
</commit_message>
<xml_diff>
--- a/Veritas_Inventory_Merged.xlsx
+++ b/Veritas_Inventory_Merged.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\nhq-inventory-portal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{699E7840-45E6-4BBB-B968-FA6D1694CC4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DCADFD2-A019-472F-80A4-092DCBD8A96E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Inventory" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Inventory!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Inventory!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="67">
   <si>
     <t>Part Number (PN)</t>
   </si>
@@ -217,18 +217,6 @@
   </si>
   <si>
     <t>Seagate Exos 7E8 4TB SAS HDD</t>
-  </si>
-  <si>
-    <t>Category</t>
-  </si>
-  <si>
-    <t>NetBackup Appliance</t>
-  </si>
-  <si>
-    <t>Other / Shared</t>
-  </si>
-  <si>
-    <t>Flex Appliance</t>
   </si>
   <si>
     <t>Quantity</t>
@@ -386,7 +374,7 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -691,41 +679,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.21875" customWidth="1"/>
     <col min="2" max="2" width="82.5546875" customWidth="1"/>
     <col min="3" max="3" width="33.21875" customWidth="1"/>
-    <col min="5" max="5" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.6640625" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" customWidth="1"/>
+    <col min="5" max="5" width="12.6640625" customWidth="1"/>
+    <col min="6" max="6" width="10.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -736,16 +720,13 @@
         <v>2</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="G2" s="3">
+        <v>66</v>
+      </c>
+      <c r="F2" s="3">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -756,16 +737,13 @@
         <v>4</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="G3" s="3">
+        <v>66</v>
+      </c>
+      <c r="F3" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -776,16 +754,13 @@
         <v>6</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="G4" s="3">
+        <v>66</v>
+      </c>
+      <c r="F4" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -796,16 +771,13 @@
         <v>8</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="G5" s="3">
+        <v>66</v>
+      </c>
+      <c r="F5" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -816,16 +788,13 @@
         <v>10</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="G6" s="3">
+        <v>66</v>
+      </c>
+      <c r="F6" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -836,16 +805,13 @@
         <v>12</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="G7" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="F7" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -856,16 +822,13 @@
         <v>14</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="G8" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="F8" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -876,16 +839,13 @@
         <v>16</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="G9" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="F9" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -896,16 +856,13 @@
         <v>18</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G10" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="F10" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -916,16 +873,13 @@
         <v>20</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="G11" s="3">
+        <v>66</v>
+      </c>
+      <c r="F11" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -936,16 +890,13 @@
         <v>22</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="G12" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="F12" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -956,16 +907,13 @@
         <v>24</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="G13" s="3">
+        <v>66</v>
+      </c>
+      <c r="F13" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -976,16 +924,13 @@
         <v>26</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="G14" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="F14" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -996,16 +941,13 @@
         <v>28</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="G15" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="F15" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -1016,16 +958,13 @@
         <v>30</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="G16" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="F16" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -1036,16 +975,13 @@
         <v>32</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="G17" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="F17" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -1056,16 +992,13 @@
         <v>34</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="G18" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="F18" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -1076,16 +1009,13 @@
         <v>36</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="G19" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="F19" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -1096,16 +1026,13 @@
         <v>38</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="G20" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="F20" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -1116,16 +1043,13 @@
         <v>40</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="G21" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="F21" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -1136,16 +1060,13 @@
         <v>42</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G22" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="F22" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -1156,16 +1077,13 @@
         <v>44</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="G23" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="F23" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -1176,16 +1094,13 @@
         <v>46</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="G24" s="3">
+        <v>66</v>
+      </c>
+      <c r="F24" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -1196,16 +1111,13 @@
         <v>48</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="G25" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="F25" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -1216,16 +1128,13 @@
         <v>50</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="G26" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="F26" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -1236,16 +1145,13 @@
         <v>52</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="G27" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="F27" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -1256,16 +1162,13 @@
         <v>54</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="G28" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="F28" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -1276,16 +1179,13 @@
         <v>56</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="G29" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="F29" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="3">
         <v>29</v>
       </c>
@@ -1296,16 +1196,13 @@
         <v>58</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="G30" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+      <c r="F30" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -1314,24 +1211,20 @@
       </c>
       <c r="C31" s="8"/>
       <c r="D31" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="G31" s="3">
+        <v>66</v>
+      </c>
+      <c r="F31" s="3">
         <v>6</v>
       </c>
     </row>
-    <row r="32" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="6"/>
       <c r="B32" s="6" t="s">
         <v>59</v>
       </c>
       <c r="C32" s="6"/>
-      <c r="E32" s="6"/>
-      <c r="G32" s="6">
-        <f>SUM(G2:G31)</f>
+      <c r="F32" s="6">
+        <f>SUM(F2:F31)</f>
         <v>50</v>
       </c>
     </row>

</xml_diff>